<commit_message>
Raise MIN_UTIL threshold to 20% and update master lorry file
A 537.8 kg load was being assigned to a 5T lorry at only 10.76%
utilisation because VEA2818 (1.07T) was already taken. Raising the
minimum utilisation threshold from 10% to 20% means a 5T lorry now
requires at least 1T of cargo; lighter loads become NO_LORRY for
manual review instead of wasting a large lorry.

VEA2818 still handles small loads (50% util for 0.54T) because
0.54T / 1.07T = 50% >> 20% threshold.

Also updates master lorry.xlsx with the latest fleet configuration.

https://claude.ai/code/session_01PiXoacUwWCUBW9ZtUd9yBt
</commit_message>
<xml_diff>
--- a/data/master lorry.xlsx
+++ b/data/master lorry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAF74F9F-459D-4EFB-823A-40508C5530D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FED6ED-E30B-4049-A651-A4FB1531209A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{400969EE-77AD-4116-B449-1FC90F02641B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="38">
   <si>
     <t>LORRY</t>
   </si>
@@ -241,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -263,6 +263,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4C2097-FE33-4A35-A59A-3B3AB0EB46A6}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -646,7 +647,7 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B28" si="0">C3/1000</f>
+        <f t="shared" ref="B3:B29" si="0">C3/1000</f>
         <v>14</v>
       </c>
       <c r="C3" s="1">
@@ -751,14 +752,14 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <v>27</v>
+      </c>
+      <c r="B9" s="11">
+        <f t="shared" ref="B9" si="1">C9/1000</f>
+        <v>8.5</v>
       </c>
       <c r="C9" s="1">
-        <v>5000</v>
+        <v>8500</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>5</v>
@@ -985,14 +986,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="B22">
-        <f t="shared" si="0"/>
-        <v>8.5</v>
+        <v>5</v>
       </c>
       <c r="C22" s="3">
-        <v>8500</v>
+        <v>5000</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>26</v>
@@ -1003,14 +1003,14 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23">
         <f t="shared" si="0"/>
-        <v>6.77</v>
+        <v>8.5</v>
       </c>
       <c r="C23" s="3">
-        <v>6770</v>
+        <v>8500</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>26</v>
@@ -1021,14 +1021,14 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6.77</v>
       </c>
       <c r="C24" s="3">
-        <v>5000</v>
+        <v>6770</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>26</v>
@@ -1038,51 +1038,51 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C25" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C26" s="4">
         <v>8000</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26">
-        <f t="shared" si="0"/>
-        <v>4.03</v>
-      </c>
-      <c r="C26" s="5">
-        <v>4030</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>3.59</v>
+        <v>4.03</v>
       </c>
       <c r="C27" s="5">
-        <v>3590</v>
+        <v>4030</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>33</v>
@@ -1093,14 +1093,14 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>3.59</v>
       </c>
       <c r="C28" s="5">
-        <v>4000</v>
+        <v>3590</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>33</v>
@@ -1109,9 +1109,27 @@
         <v>37</v>
       </c>
     </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C29" s="5">
+        <v>4000</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E28" xr:uid="{58B93DB1-8C6E-43BC-8022-F0886421921B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E29" xr:uid="{58B93DB1-8C6E-43BC-8022-F0886421921B}">
       <formula1>"Available, Block"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>